<commit_message>
data: actualizacion automatica 2026-06-19
</commit_message>
<xml_diff>
--- a/data/estadisticas_poblacion_2026-06-19.xlsx
+++ b/data/estadisticas_poblacion_2026-06-19.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-19 16:00 UTC</t>
+          <t>2026-06-19 16:29 UTC</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>Sub-Saharan Africa (IDA &amp; IBRD countries)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SSF</t>
+          <t>TSS</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -970,12 +970,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa (IDA &amp; IBRD countries)</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TSS</t>
+          <t>SSF</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -43912,12 +43912,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sint Maarten (Dutch part)</t>
+          <t>Bahrain</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SXM</t>
+          <t>BHR</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -43927,21 +43927,21 @@
         <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>1.4</v>
+        <v>0.73</v>
       </c>
       <c r="F2" t="n">
-        <v>558</v>
+        <v>22699</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>BMU</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -43951,21 +43951,21 @@
         <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>1.99</v>
+        <v>-0.1</v>
       </c>
       <c r="F3" t="n">
-        <v>20011</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cayman Islands</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYM</t>
+          <t>SGP</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -43975,21 +43975,21 @@
         <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>1.92</v>
+        <v>1.99</v>
       </c>
       <c r="F4" t="n">
-        <v>896</v>
+        <v>20011</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nauru</t>
+          <t>Sint Maarten (Dutch part)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NRU</t>
+          <t>SXM</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -43999,21 +43999,21 @@
         <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="F5" t="n">
-        <v>-121</v>
+        <v>558</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>St. Martin (French part)</t>
+          <t>Cayman Islands</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MAF</t>
+          <t>CYM</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -44023,21 +44023,21 @@
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>-5.17</v>
+        <v>1.92</v>
       </c>
       <c r="F6" t="n">
-        <v>-1424</v>
+        <v>896</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gibraltar</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GIB</t>
+          <t>MCO</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -44047,21 +44047,21 @@
         <v>100</v>
       </c>
       <c r="E7" t="n">
-        <v>2.21</v>
+        <v>-0.84</v>
       </c>
       <c r="F7" t="n">
-        <v>598</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hong Kong SAR, China</t>
+          <t>St. Martin (French part)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MAF</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -44071,21 +44071,21 @@
         <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.16</v>
+        <v>-5.17</v>
       </c>
       <c r="F8" t="n">
-        <v>-19272</v>
+        <v>-1424</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>Nauru</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BHR</t>
+          <t>NRU</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -44095,21 +44095,21 @@
         <v>100</v>
       </c>
       <c r="E9" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="F9" t="n">
-        <v>22699</v>
+        <v>-121</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Macao SAR, China</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BMU</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -44119,21 +44119,21 @@
         <v>100</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1</v>
+        <v>1.2</v>
       </c>
       <c r="F10" t="n">
-        <v>-5</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Macao SAR, China</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MAC</t>
+          <t>KWT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -44143,21 +44143,21 @@
         <v>100</v>
       </c>
       <c r="E11" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="F11" t="n">
-        <v>1620</v>
+        <v>61624</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Gibraltar</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KWT</t>
+          <t>GIB</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -44167,21 +44167,21 @@
         <v>100</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9</v>
+        <v>2.21</v>
       </c>
       <c r="F12" t="n">
-        <v>61624</v>
+        <v>598</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Hong Kong SAR, China</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -44191,10 +44191,10 @@
         <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.84</v>
+        <v>-0.16</v>
       </c>
       <c r="F13" t="n">
-        <v>110</v>
+        <v>-19272</v>
       </c>
     </row>
     <row r="14">
@@ -45184,12 +45184,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Latin America &amp; the Caribbean (IDA &amp; IBRD countries)</t>
+          <t>Latin America &amp; Caribbean</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TLA</t>
+          <t>LCN</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -45199,21 +45199,21 @@
         <v>81.27</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="F55" t="n">
-        <v>-369248</v>
+        <v>-378373</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Latin America &amp; Caribbean</t>
+          <t>Latin America &amp; the Caribbean (IDA &amp; IBRD countries)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LCN</t>
+          <t>TLA</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -45223,10 +45223,10 @@
         <v>81.27</v>
       </c>
       <c r="E56" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>-378373</v>
+        <v>-369248</v>
       </c>
     </row>
     <row r="57">
@@ -49312,12 +49312,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Tanzania</t>
+          <t>Least developed countries: UN classification</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>TZA</t>
+          <t>LDC</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -49327,21 +49327,21 @@
         <v>36.17</v>
       </c>
       <c r="E227" t="n">
-        <v>4.81</v>
+        <v>3.6</v>
       </c>
       <c r="F227" t="n">
-        <v>-29865</v>
+        <v>-1748381</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Least developed countries: UN classification</t>
+          <t>Tanzania</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>LDC</t>
+          <t>TZA</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -49351,10 +49351,10 @@
         <v>36.17</v>
       </c>
       <c r="E228" t="n">
-        <v>3.6</v>
+        <v>4.81</v>
       </c>
       <c r="F228" t="n">
-        <v>-1748381</v>
+        <v>-29865</v>
       </c>
     </row>
     <row r="229">

</xml_diff>